<commit_message>
cambios en el excel
</commit_message>
<xml_diff>
--- a/backend/database/Seguidores_Segundo_Modulo.xlsx
+++ b/backend/database/Seguidores_Segundo_Modulo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24b0972e82577483/CLOUDGER/DOCKER/NOTAS_MOVI_APP/notasseguidores/app/backend/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{EBDF6B2D-AFF0-4FB6-A7CB-8EBDF6A593F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34AE2D8D-5EED-4EDC-ADE8-B097BE201AFB}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{EBDF6B2D-AFF0-4FB6-A7CB-8EBDF6A593F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BBA3B3E-9F88-4974-B1BE-389FFC4B23A0}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{69E08A24-6B7F-4298-AF10-6623656F96D4}"/>
   </bookViews>
@@ -2195,7 +2195,7 @@
         <v>10</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K2">
         <v>10</v>
@@ -2213,7 +2213,7 @@
         <v>10</v>
       </c>
       <c r="P2">
-        <f>ROUNDUP(AVERAGE(D2:O2),0)</f>
+        <f>ROUND(AVERAGE(D2:O2),0)</f>
         <v>10</v>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
         <v>10</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K3">
         <v>10</v>
@@ -2264,7 +2264,7 @@
         <v>10</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P65" si="0">ROUNDUP(AVERAGE(D3:O3),0)</f>
+        <f t="shared" ref="P3:Q66" si="0">ROUND(AVERAGE(D3:O3),0)</f>
         <v>10</v>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
         <v>10</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K4">
         <v>10</v>
@@ -2348,7 +2348,7 @@
         <v>10</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K5">
         <v>10</v>
@@ -2399,7 +2399,7 @@
         <v>10</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K6">
         <v>10</v>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="P6">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -2450,7 +2450,7 @@
         <v>10</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K7">
         <v>10</v>
@@ -2501,7 +2501,7 @@
         <v>0</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K8">
         <v>10</v>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="P8">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -2603,7 +2603,7 @@
         <v>10</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K10">
         <v>10</v>
@@ -2654,7 +2654,7 @@
         <v>10</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -2705,7 +2705,7 @@
         <v>10</v>
       </c>
       <c r="J12">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K12">
         <v>10</v>
@@ -2756,7 +2756,7 @@
         <v>10</v>
       </c>
       <c r="J13">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K13">
         <v>10</v>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="P13">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -2807,7 +2807,7 @@
         <v>10</v>
       </c>
       <c r="J14">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K14">
         <v>10</v>
@@ -2858,7 +2858,7 @@
         <v>10</v>
       </c>
       <c r="J15">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K15">
         <v>10</v>
@@ -2909,7 +2909,7 @@
         <v>0</v>
       </c>
       <c r="J16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K16">
         <v>10</v>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="P16">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
@@ -2960,7 +2960,7 @@
         <v>10</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K17">
         <v>10</v>
@@ -3011,7 +3011,7 @@
         <v>10</v>
       </c>
       <c r="J18">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K18">
         <v>10</v>
@@ -3062,7 +3062,7 @@
         <v>0</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K19">
         <v>10</v>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="P19">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
@@ -3113,7 +3113,7 @@
         <v>0</v>
       </c>
       <c r="J20">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K20">
         <v>10</v>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="P20">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
@@ -3164,7 +3164,7 @@
         <v>10</v>
       </c>
       <c r="J21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -3215,7 +3215,7 @@
         <v>10</v>
       </c>
       <c r="J22">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="P22">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
@@ -3266,7 +3266,7 @@
         <v>10</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K23">
         <v>10</v>
@@ -3317,7 +3317,7 @@
         <v>0</v>
       </c>
       <c r="J24">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K24">
         <v>10</v>
@@ -3368,7 +3368,7 @@
         <v>10</v>
       </c>
       <c r="J25">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K25">
         <v>10</v>
@@ -3419,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="J26">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="P26">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
@@ -3470,7 +3470,7 @@
         <v>10</v>
       </c>
       <c r="J27">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K27">
         <v>10</v>
@@ -3521,7 +3521,7 @@
         <v>10</v>
       </c>
       <c r="J28">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K28">
         <v>10</v>
@@ -3572,7 +3572,7 @@
         <v>10</v>
       </c>
       <c r="J29">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K29">
         <v>10</v>
@@ -3623,7 +3623,7 @@
         <v>10</v>
       </c>
       <c r="J30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K30">
         <v>10</v>
@@ -3674,7 +3674,7 @@
         <v>10</v>
       </c>
       <c r="J31">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K31">
         <v>10</v>
@@ -3725,7 +3725,7 @@
         <v>10</v>
       </c>
       <c r="J32">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -3776,7 +3776,7 @@
         <v>0</v>
       </c>
       <c r="J33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K33">
         <v>10</v>
@@ -3827,7 +3827,7 @@
         <v>10</v>
       </c>
       <c r="J34">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K34">
         <v>10</v>
@@ -3878,7 +3878,7 @@
         <v>10</v>
       </c>
       <c r="J35">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K35">
         <v>10</v>
@@ -3929,7 +3929,7 @@
         <v>10</v>
       </c>
       <c r="J36">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K36">
         <v>10</v>
@@ -3980,7 +3980,7 @@
         <v>10</v>
       </c>
       <c r="J37">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K37">
         <v>10</v>
@@ -4031,7 +4031,7 @@
         <v>0</v>
       </c>
       <c r="J38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K38">
         <v>10</v>
@@ -4082,7 +4082,7 @@
         <v>10</v>
       </c>
       <c r="J39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K39">
         <v>10</v>
@@ -4130,7 +4130,7 @@
         <v>10</v>
       </c>
       <c r="J40">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K40">
         <v>10</v>
@@ -4181,7 +4181,7 @@
         <v>10</v>
       </c>
       <c r="J41">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K41">
         <v>10</v>
@@ -4232,7 +4232,7 @@
         <v>0</v>
       </c>
       <c r="J42">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="P42">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
@@ -4283,7 +4283,7 @@
         <v>10</v>
       </c>
       <c r="J43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K43">
         <v>10</v>
@@ -4334,7 +4334,7 @@
         <v>10</v>
       </c>
       <c r="J44">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K44">
         <v>10</v>
@@ -4385,7 +4385,7 @@
         <v>10</v>
       </c>
       <c r="J45">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K45">
         <v>10</v>
@@ -4436,7 +4436,7 @@
         <v>0</v>
       </c>
       <c r="J46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K46">
         <v>10</v>
@@ -4487,7 +4487,7 @@
         <v>10</v>
       </c>
       <c r="J47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K47">
         <v>10</v>
@@ -4538,7 +4538,7 @@
         <v>10</v>
       </c>
       <c r="J48">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K48">
         <v>10</v>
@@ -4589,7 +4589,7 @@
         <v>10</v>
       </c>
       <c r="J49">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K49">
         <v>10</v>
@@ -4640,7 +4640,7 @@
         <v>10</v>
       </c>
       <c r="J50">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K50">
         <v>10</v>
@@ -4691,7 +4691,7 @@
         <v>0</v>
       </c>
       <c r="J51">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K51">
         <v>10</v>
@@ -4742,7 +4742,7 @@
         <v>10</v>
       </c>
       <c r="J52">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K52">
         <v>10</v>
@@ -4793,7 +4793,7 @@
         <v>0</v>
       </c>
       <c r="J53">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K53">
         <v>10</v>
@@ -4812,7 +4812,7 @@
       </c>
       <c r="P53">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
@@ -4844,7 +4844,7 @@
         <v>0</v>
       </c>
       <c r="J54">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K54">
         <v>0</v>
@@ -4863,7 +4863,7 @@
       </c>
       <c r="P54">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
@@ -4895,7 +4895,7 @@
         <v>10</v>
       </c>
       <c r="J55">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K55">
         <v>0</v>
@@ -4946,7 +4946,7 @@
         <v>10</v>
       </c>
       <c r="J56">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K56">
         <v>10</v>
@@ -4997,7 +4997,7 @@
         <v>10</v>
       </c>
       <c r="J57">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K57">
         <v>0</v>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="P57">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>0</v>
       </c>
       <c r="J58">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="P58">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
@@ -5099,7 +5099,7 @@
         <v>10</v>
       </c>
       <c r="J59">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K59">
         <v>10</v>
@@ -5150,7 +5150,7 @@
         <v>10</v>
       </c>
       <c r="J60">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K60">
         <v>10</v>
@@ -5201,7 +5201,7 @@
         <v>10</v>
       </c>
       <c r="J61">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K61">
         <v>10</v>
@@ -5252,7 +5252,7 @@
         <v>10</v>
       </c>
       <c r="J62">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K62">
         <v>10</v>
@@ -5303,7 +5303,7 @@
         <v>10</v>
       </c>
       <c r="J63">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K63">
         <v>10</v>
@@ -5354,7 +5354,7 @@
         <v>10</v>
       </c>
       <c r="J64">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K64">
         <v>10</v>
@@ -5405,7 +5405,7 @@
         <v>10</v>
       </c>
       <c r="J65">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K65">
         <v>10</v>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="P65">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
@@ -5474,8 +5474,8 @@
         <v>10</v>
       </c>
       <c r="P66">
-        <f t="shared" ref="P66:P129" si="1">ROUNDUP(AVERAGE(D66:O66),0)</f>
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
@@ -5507,7 +5507,7 @@
         <v>10</v>
       </c>
       <c r="J67">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K67">
         <v>0</v>
@@ -5525,7 +5525,7 @@
         <v>0</v>
       </c>
       <c r="P67">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="P67:P130" si="1">ROUND(AVERAGE(D67:O67),0)</f>
         <v>5</v>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
         <v>0</v>
       </c>
       <c r="J68">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K68">
         <v>10</v>
@@ -5577,7 +5577,7 @@
       </c>
       <c r="P68">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
@@ -5609,7 +5609,7 @@
         <v>0</v>
       </c>
       <c r="J69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K69">
         <v>10</v>
@@ -5628,7 +5628,7 @@
       </c>
       <c r="P69">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
@@ -5660,7 +5660,7 @@
         <v>10</v>
       </c>
       <c r="J70">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K70">
         <v>10</v>
@@ -5711,7 +5711,7 @@
         <v>10</v>
       </c>
       <c r="J71">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K71">
         <v>10</v>
@@ -5762,7 +5762,7 @@
         <v>10</v>
       </c>
       <c r="J72">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K72">
         <v>10</v>
@@ -5813,7 +5813,7 @@
         <v>0</v>
       </c>
       <c r="J73">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K73">
         <v>10</v>
@@ -5832,7 +5832,7 @@
       </c>
       <c r="P73">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
@@ -5864,7 +5864,7 @@
         <v>10</v>
       </c>
       <c r="J74">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K74">
         <v>10</v>
@@ -5915,7 +5915,7 @@
         <v>10</v>
       </c>
       <c r="J75">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K75">
         <v>10</v>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="P77">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
@@ -6068,7 +6068,7 @@
         <v>0</v>
       </c>
       <c r="J78">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K78">
         <v>10</v>
@@ -6119,7 +6119,7 @@
         <v>10</v>
       </c>
       <c r="J79">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K79">
         <v>10</v>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="P79">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.25">
@@ -6170,7 +6170,7 @@
         <v>10</v>
       </c>
       <c r="J80">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K80">
         <v>10</v>
@@ -6221,7 +6221,7 @@
         <v>10</v>
       </c>
       <c r="J81">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K81">
         <v>10</v>
@@ -6272,7 +6272,7 @@
         <v>10</v>
       </c>
       <c r="J82">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K82">
         <v>10</v>
@@ -6291,7 +6291,7 @@
       </c>
       <c r="P82">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
@@ -6323,7 +6323,7 @@
         <v>0</v>
       </c>
       <c r="J83">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K83">
         <v>10</v>
@@ -6374,7 +6374,7 @@
         <v>10</v>
       </c>
       <c r="J84">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K84">
         <v>10</v>
@@ -6425,7 +6425,7 @@
         <v>10</v>
       </c>
       <c r="J85">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K85">
         <v>10</v>
@@ -6476,7 +6476,7 @@
         <v>10</v>
       </c>
       <c r="J86">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K86">
         <v>10</v>
@@ -6527,7 +6527,7 @@
         <v>10</v>
       </c>
       <c r="J87">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K87">
         <v>10</v>
@@ -6578,7 +6578,7 @@
         <v>10</v>
       </c>
       <c r="J88">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K88">
         <v>10</v>
@@ -6629,7 +6629,7 @@
         <v>10</v>
       </c>
       <c r="J89">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K89">
         <v>10</v>
@@ -6648,7 +6648,7 @@
       </c>
       <c r="P89">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90" spans="1:16" x14ac:dyDescent="0.25">
@@ -6680,7 +6680,7 @@
         <v>10</v>
       </c>
       <c r="J90">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K90">
         <v>10</v>
@@ -6731,7 +6731,7 @@
         <v>10</v>
       </c>
       <c r="J91">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K91">
         <v>10</v>
@@ -6782,7 +6782,7 @@
         <v>10</v>
       </c>
       <c r="J92">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K92">
         <v>10</v>
@@ -6833,7 +6833,7 @@
         <v>10</v>
       </c>
       <c r="J93">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K93">
         <v>10</v>
@@ -6884,7 +6884,7 @@
         <v>0</v>
       </c>
       <c r="J94">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K94">
         <v>10</v>
@@ -7037,7 +7037,7 @@
         <v>10</v>
       </c>
       <c r="J97">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K97">
         <v>10</v>
@@ -7088,7 +7088,7 @@
         <v>10</v>
       </c>
       <c r="J98">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K98">
         <v>10</v>
@@ -7139,7 +7139,7 @@
         <v>0</v>
       </c>
       <c r="J99">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K99">
         <v>10</v>
@@ -7190,7 +7190,7 @@
         <v>10</v>
       </c>
       <c r="J100">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K100">
         <v>10</v>
@@ -7209,7 +7209,7 @@
       </c>
       <c r="P100">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="101" spans="1:16" x14ac:dyDescent="0.25">
@@ -7241,7 +7241,7 @@
         <v>10</v>
       </c>
       <c r="J101">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K101">
         <v>10</v>
@@ -7292,7 +7292,7 @@
         <v>10</v>
       </c>
       <c r="J102">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K102">
         <v>10</v>
@@ -7343,7 +7343,7 @@
         <v>10</v>
       </c>
       <c r="J103">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K103">
         <v>10</v>
@@ -7394,7 +7394,7 @@
         <v>10</v>
       </c>
       <c r="J104">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K104">
         <v>10</v>
@@ -7445,7 +7445,7 @@
         <v>0</v>
       </c>
       <c r="J105">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K105">
         <v>0</v>
@@ -7496,7 +7496,7 @@
         <v>10</v>
       </c>
       <c r="J106">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K106">
         <v>10</v>
@@ -7547,7 +7547,7 @@
         <v>10</v>
       </c>
       <c r="J107">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K107">
         <v>0</v>
@@ -7566,7 +7566,7 @@
       </c>
       <c r="P107">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="108" spans="1:16" x14ac:dyDescent="0.25">
@@ -7595,7 +7595,7 @@
         <v>0</v>
       </c>
       <c r="J108">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K108">
         <v>10</v>
@@ -7614,7 +7614,7 @@
       </c>
       <c r="P108">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="109" spans="1:16" x14ac:dyDescent="0.25">
@@ -7646,7 +7646,7 @@
         <v>10</v>
       </c>
       <c r="J109">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K109">
         <v>10</v>
@@ -7697,7 +7697,7 @@
         <v>10</v>
       </c>
       <c r="J110">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K110">
         <v>10</v>
@@ -7716,7 +7716,7 @@
       </c>
       <c r="P110">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="111" spans="1:16" x14ac:dyDescent="0.25">
@@ -7748,7 +7748,7 @@
         <v>10</v>
       </c>
       <c r="J111">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K111">
         <v>0</v>
@@ -7799,7 +7799,7 @@
         <v>10</v>
       </c>
       <c r="J112">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K112">
         <v>10</v>
@@ -7850,7 +7850,7 @@
         <v>0</v>
       </c>
       <c r="J113">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K113">
         <v>10</v>
@@ -7869,7 +7869,7 @@
       </c>
       <c r="P113">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114" spans="1:16" x14ac:dyDescent="0.25">
@@ -7901,7 +7901,7 @@
         <v>10</v>
       </c>
       <c r="J114">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K114">
         <v>10</v>
@@ -7952,7 +7952,7 @@
         <v>10</v>
       </c>
       <c r="J115">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K115">
         <v>10</v>
@@ -8003,7 +8003,7 @@
         <v>10</v>
       </c>
       <c r="J116">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K116">
         <v>10</v>
@@ -8054,7 +8054,7 @@
         <v>10</v>
       </c>
       <c r="J117">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K117">
         <v>10</v>
@@ -8105,7 +8105,7 @@
         <v>10</v>
       </c>
       <c r="J118">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K118">
         <v>10</v>
@@ -8156,7 +8156,7 @@
         <v>10</v>
       </c>
       <c r="J119">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K119">
         <v>10</v>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="P119">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="120" spans="1:16" x14ac:dyDescent="0.25">
@@ -8207,7 +8207,7 @@
         <v>0</v>
       </c>
       <c r="J120">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K120">
         <v>0</v>
@@ -8226,7 +8226,7 @@
       </c>
       <c r="P120">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121" spans="1:16" x14ac:dyDescent="0.25">
@@ -8258,7 +8258,7 @@
         <v>10</v>
       </c>
       <c r="J121">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K121">
         <v>10</v>
@@ -8309,7 +8309,7 @@
         <v>0</v>
       </c>
       <c r="J122">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K122">
         <v>10</v>
@@ -8328,7 +8328,7 @@
       </c>
       <c r="P122">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="123" spans="1:16" x14ac:dyDescent="0.25">
@@ -8360,7 +8360,7 @@
         <v>10</v>
       </c>
       <c r="J123">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K123">
         <v>10</v>
@@ -8411,7 +8411,7 @@
         <v>10</v>
       </c>
       <c r="J124">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K124">
         <v>0</v>
@@ -8462,7 +8462,7 @@
         <v>10</v>
       </c>
       <c r="J125">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K125">
         <v>10</v>
@@ -8513,7 +8513,7 @@
         <v>10</v>
       </c>
       <c r="J126">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K126">
         <v>10</v>
@@ -8564,7 +8564,7 @@
         <v>10</v>
       </c>
       <c r="J127">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K127">
         <v>10</v>
@@ -8615,7 +8615,7 @@
         <v>10</v>
       </c>
       <c r="J128">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K128">
         <v>0</v>
@@ -8666,7 +8666,7 @@
         <v>10</v>
       </c>
       <c r="J129">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K129">
         <v>10</v>
@@ -8717,7 +8717,7 @@
         <v>10</v>
       </c>
       <c r="J130">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K130">
         <v>10</v>
@@ -8735,7 +8735,7 @@
         <v>0</v>
       </c>
       <c r="P130">
-        <f t="shared" ref="P130:P139" si="2">ROUNDUP(AVERAGE(D130:O130),0)</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -8768,7 +8768,7 @@
         <v>10</v>
       </c>
       <c r="J131">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K131">
         <v>0</v>
@@ -8786,7 +8786,7 @@
         <v>10</v>
       </c>
       <c r="P131">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="P131:P139" si="2">ROUND(AVERAGE(D131:O131),0)</f>
         <v>8</v>
       </c>
     </row>
@@ -8819,7 +8819,7 @@
         <v>0</v>
       </c>
       <c r="J132">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K132">
         <v>10</v>
@@ -8838,7 +8838,7 @@
       </c>
       <c r="P132">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="133" spans="1:16" x14ac:dyDescent="0.25">
@@ -8870,7 +8870,7 @@
         <v>10</v>
       </c>
       <c r="J133">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K133">
         <v>10</v>
@@ -8921,7 +8921,7 @@
         <v>10</v>
       </c>
       <c r="J134">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K134">
         <v>10</v>
@@ -8972,7 +8972,7 @@
         <v>10</v>
       </c>
       <c r="J135">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K135">
         <v>10</v>
@@ -9023,7 +9023,7 @@
         <v>10</v>
       </c>
       <c r="J136">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K136">
         <v>10</v>
@@ -9074,7 +9074,7 @@
         <v>10</v>
       </c>
       <c r="J137">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K137">
         <v>10</v>
@@ -9125,7 +9125,7 @@
         <v>0</v>
       </c>
       <c r="J138">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K138">
         <v>10</v>
@@ -9176,7 +9176,7 @@
         <v>0</v>
       </c>
       <c r="J139">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K139">
         <v>0</v>
@@ -9195,7 +9195,7 @@
       </c>
       <c r="P139">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>